<commit_message>
Use day1/day2/day4 Excel sheet names
Standardize exported weekday labels as day1 (Monday), day2 (Tuesday), and day4 (Thursday), and update the documentation and cycle workbooks to match.
</commit_message>
<xml_diff>
--- a/results/reservation_cycle32_20260906.xlsx
+++ b/results/reservation_cycle32_20260906.xlsx
@@ -13,9 +13,9 @@
     <workbookView xWindow="5500" yWindow="660" windowWidth="26660" windowHeight="15640" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="mon" sheetId="1" r:id="rId1"/>
-    <sheet name="tue" sheetId="2" r:id="rId2"/>
-    <sheet name="thur" sheetId="3" r:id="rId3"/>
+    <sheet name="day1" sheetId="1" r:id="rId1"/>
+    <sheet name="day2" sheetId="2" r:id="rId2"/>
+    <sheet name="day4" sheetId="3" r:id="rId3"/>
     <sheet name="Summary" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -52,7 +52,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>mon</t>
+    <t>day1</t>
   </si>
   <si>
     <t>00:00~02:00</t>
@@ -391,7 +391,7 @@
     <t>Preferred time (UTC)</t>
   </si>
   <si>
-    <t>tue</t>
+    <t>day2</t>
   </si>
   <si>
     <t>SirMike</t>
@@ -421,28 +421,28 @@
     <t>Viiii</t>
   </si>
   <si>
-    <t>thur</t>
+    <t>day4</t>
   </si>
   <si>
     <t>WiessVV</t>
   </si>
   <si>
-    <t>mon Players</t>
-  </si>
-  <si>
-    <t>mon Speedup</t>
-  </si>
-  <si>
-    <t>tue Players</t>
-  </si>
-  <si>
-    <t>tue Speedup</t>
-  </si>
-  <si>
-    <t>thur Players</t>
-  </si>
-  <si>
-    <t>thur Speedup</t>
+    <t>day1 Players</t>
+  </si>
+  <si>
+    <t>day1 Speedup</t>
+  </si>
+  <si>
+    <t>day2 Players</t>
+  </si>
+  <si>
+    <t>day2 Speedup</t>
+  </si>
+  <si>
+    <t>day4 Players</t>
+  </si>
+  <si>
+    <t>day4 Speedup</t>
   </si>
   <si>
     <t>Total Players</t>

</xml_diff>